<commit_message>
A programme is its head and its code; panel and page now agree everywhere
</commit_message>
<xml_diff>
--- a/brunei/FINAL_PANEL.xlsx
+++ b/brunei/FINAL_PANEL.xlsx
@@ -9508,11 +9508,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Development of school and higher education institution infrastructure under the 12th National Development Plan; Focus projects to support the budget focus areas for Financial Year 2024/2025; MPEC programmes: i-Ready, TVET Scheme, Skillsplus, SPIN in Accountancy and Tradeskills; Miftaahun Najaah Scheme; Research and innovation allocations under the 12th National Development Plan; Research costs for public higher education institutions; Scholarships through the Ministry of Education and the Ministry of Religious Affairs</t>
-        </is>
-      </c>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9586,11 +9582,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Development of school and higher education institution infrastructure under the 12th National Development Plan; Focus projects to support the budget focus areas for Financial Year 2024/2025</t>
-        </is>
-      </c>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9664,11 +9656,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Electricity supply projects under the 12th National Development Plan; Green Building initiatives under the 12th National Development Plan</t>
-        </is>
-      </c>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9742,11 +9730,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Electricity supply projects under the 12th National Development Plan</t>
-        </is>
-      </c>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9820,11 +9804,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>National housing provision projects under the 12th National Development Plan</t>
-        </is>
-      </c>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9898,11 +9878,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Water supply and sewerage system upgrading projects under the 12th National Development Plan</t>
-        </is>
-      </c>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9976,11 +9952,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>Medical and health infrastructure development under the 12th National Development Plan</t>
-        </is>
-      </c>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -10042,11 +10014,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Payment for medical treatment services at Gleneagles Jerudong Park Medical Centre, Brunei Cancer Centre and Brunei Neuroscience, Stroke and Rehabilitation Centre</t>
-        </is>
-      </c>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -10120,11 +10088,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>IT Central Procurement projects and software licences for all ministries and government departments</t>
-        </is>
-      </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -10198,11 +10162,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>Aquaculture industry site development and basic infrastructure projects; Infrastructure provision for enhancement of the agricultural industry nationwide - Phase 2; Livestock industry development plan; Preparation and upgrading works for infrastructure and basic facilities in existing and new agricultural development areas</t>
-        </is>
-      </c>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -10276,11 +10236,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>Infrastructure provision for enhancement of the agricultural industry nationwide - Phase 2; Preparation and upgrading works for infrastructure and basic facilities in existing and new agricultural development areas</t>
-        </is>
-      </c>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -10354,11 +10310,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>Focus projects to support the budget focus areas for Financial Year 2024/2025; Research and innovation allocations under the 12th National Development Plan</t>
-        </is>
-      </c>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -10420,11 +10372,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>Purchase of medicines, medical consumables and laboratory testing needs</t>
-        </is>
-      </c>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -10498,11 +10446,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>Bru-HIMS 2.0 system project; Maintenance of Bru-HIMS and enhancement of BruHealth system features</t>
-        </is>
-      </c>
+      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -10576,11 +10520,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>Capacity enhancement programme for irrigation systems in agricultural development areas nationwide - Phase 2; Preparation and upgrading works for infrastructure and basic facilities in existing and new agricultural development areas</t>
-        </is>
-      </c>
+      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -10654,11 +10594,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>Focus projects to support the budget focus areas for Financial Year 2024/2025; Scholarships through the Ministry of Education and the Ministry of Religious Affairs</t>
-        </is>
-      </c>
+      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -10732,11 +10668,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>Flood prevention projects under the 12th National Development Plan</t>
-        </is>
-      </c>
+      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10810,11 +10742,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>Airport infrastructure modernisation projects under the 12th National Development Plan</t>
-        </is>
-      </c>
+      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -10888,11 +10816,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>Education digital infrastructure and smart systems under the 12th National Development Plan; Focus projects to support the budget focus areas for Financial Year 2024/2025</t>
-        </is>
-      </c>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -10966,11 +10890,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>Focus projects to support the budget focus areas for Financial Year 2024/2025; MPEC programmes: i-Ready, TVET Scheme, Skillsplus, SPIN in Accountancy and Tradeskills</t>
-        </is>
-      </c>
+      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -11044,11 +10964,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>Education information and data management systems under the 12th National Development Plan; Focus projects to support the budget focus areas for Financial Year 2024/2025</t>
-        </is>
-      </c>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -11122,11 +11038,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>Management of infectious disease crises and assistance to affected individuals or communities</t>
-        </is>
-      </c>
+      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -11200,11 +11112,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>Government digital transformation projects under the 12th National Development Plan</t>
-        </is>
-      </c>
+      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -11278,11 +11186,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>Tourism product improvement projects under the 12th National Development Plan</t>
-        </is>
-      </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -11356,11 +11260,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>Integrated government databases and asset management systems under the 12th National Development Plan</t>
-        </is>
-      </c>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -11434,11 +11334,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>Focus projects to support the budget focus areas for Financial Year 2024/2025; Miftaahun Najaah Scheme</t>
-        </is>
-      </c>
+      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -11512,11 +11408,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>High-technology vegetable production enhancement programme under the 12th National Development Plan; Preparation and upgrading works for infrastructure and basic facilities in existing and new agricultural development areas</t>
-        </is>
-      </c>
+      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -11590,11 +11482,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>Focus projects to support the budget focus areas for Financial Year 2024/2025</t>
-        </is>
-      </c>
+      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -11668,11 +11556,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>Focus projects to support the budget focus areas for Financial Year 2024/2025</t>
-        </is>
-      </c>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -11746,11 +11630,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>Focus projects to support the budget focus areas for Financial Year 2024/2025</t>
-        </is>
-      </c>
+      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -11824,11 +11704,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>Quality health service support provision</t>
-        </is>
-      </c>
+      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -11902,11 +11778,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>Maintenance of Bru-HIMS and enhancement of BruHealth system features</t>
-        </is>
-      </c>
+      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -11980,11 +11852,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>Natural disaster management</t>
-        </is>
-      </c>
+      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -12046,11 +11914,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>Judiciary digital case management systems under the 12th National Development Plan</t>
-        </is>
-      </c>
+      <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -12112,11 +11976,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>Aquaculture industry site development and basic infrastructure projects</t>
-        </is>
-      </c>
+      <c r="P36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -12190,11 +12050,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>Livestock industry development plan</t>
-        </is>
-      </c>
+      <c r="P37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -12268,11 +12124,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>Environmental sustainability, reforestation and forest conservation programmes under the 12th National Development Plan</t>
-        </is>
-      </c>
+      <c r="P38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -12346,11 +12198,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>Digital transformation in the transport and logistics sector under the 12th National Development Plan</t>
-        </is>
-      </c>
+      <c r="P39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -12424,11 +12272,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>Migration from TAFIS 1.0 to TAFIS 2.0</t>
-        </is>
-      </c>
+      <c r="P40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -12490,11 +12334,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t>Preparation and upgrading works for infrastructure and basic facilities in existing and new agricultural development areas</t>
-        </is>
-      </c>
+      <c r="P41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -12556,11 +12396,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>Paddy buy-back scheme and purchase of hybrid paddy seeds</t>
-        </is>
-      </c>
+      <c r="P42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -12634,11 +12470,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>Research costs for public higher education institutions</t>
-        </is>
-      </c>
+      <c r="P43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -12712,11 +12544,7 @@
           <t>BND million</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>National Adaptation Plan for Climate Change under the 12th National Development Plan</t>
-        </is>
-      </c>
+      <c r="P44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">

</xml_diff>